<commit_message>
Reading and Writing excel Data- eform6
</commit_message>
<xml_diff>
--- a/src/test/resources/data/BAT/testData.xlsx
+++ b/src/test/resources/data/BAT/testData.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wsib-my.sharepoint.com/personal/kiran_kangula_wsib_on_ca/Documents/Documents/Automation/DigitalClaims/src/test/resources/data/BAT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="11_F25DC773A252ABDACC104813615A72165ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81F76BF5-7120-478E-8F09-664D83C3CCE9}"/>
+  <xr:revisionPtr revIDLastSave="74" documentId="11_F25DC773A252ABDACC104821899F6F185BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C923FAD-C4A3-4049-BCE3-78BA9DC4B86A}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GWCC" sheetId="1" r:id="rId1"/>
+    <sheet name="eForm6" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,30 +37,150 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
-  <si>
-    <t>PIN</t>
-  </si>
-  <si>
-    <t>DOB</t>
-  </si>
-  <si>
-    <t>Claim Number</t>
-  </si>
-  <si>
-    <t>859275</t>
-  </si>
-  <si>
-    <t>01/Jan/2000</t>
-  </si>
-  <si>
-    <t>32650342</t>
-  </si>
-  <si>
-    <t>903421</t>
-  </si>
-  <si>
-    <t>32650343</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="48">
+  <si>
+    <t>ReferenceNumber</t>
+  </si>
+  <si>
+    <t>ReportType</t>
+  </si>
+  <si>
+    <t>InjuryType</t>
+  </si>
+  <si>
+    <t>PhysicalInjury</t>
+  </si>
+  <si>
+    <t>BodyPart</t>
+  </si>
+  <si>
+    <t>ExistingClaimNumber</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>PhoneNumber</t>
+  </si>
+  <si>
+    <t>Pronouns</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>DateofBirthDay</t>
+  </si>
+  <si>
+    <t>DateofBirthMonth</t>
+  </si>
+  <si>
+    <t>DateofBirthYear</t>
+  </si>
+  <si>
+    <t>sinNumber</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>Province</t>
+  </si>
+  <si>
+    <t>PostalCode</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>EmployerName</t>
+  </si>
+  <si>
+    <t>EmployerAddress</t>
+  </si>
+  <si>
+    <t>EmployerCity</t>
+  </si>
+  <si>
+    <t>EmployerProvince</t>
+  </si>
+  <si>
+    <t>EmployerPostalCode</t>
+  </si>
+  <si>
+    <t>EmployerCountry</t>
+  </si>
+  <si>
+    <t>Injury or Illness</t>
+  </si>
+  <si>
+    <t>Physical Injury</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Burn</t>
+  </si>
+  <si>
+    <t>Kiran</t>
+  </si>
+  <si>
+    <t>Kangula</t>
+  </si>
+  <si>
+    <t>6478888888</t>
+  </si>
+  <si>
+    <t>He/Him</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>2000</t>
+  </si>
+  <si>
+    <t>English</t>
+  </si>
+  <si>
+    <t>140 Erskine Ave</t>
+  </si>
+  <si>
+    <t>Toronto</t>
+  </si>
+  <si>
+    <t>Ontario</t>
+  </si>
+  <si>
+    <t>M4P 1Z2</t>
+  </si>
+  <si>
+    <t>Canada</t>
+  </si>
+  <si>
+    <t>TestEmpl</t>
+  </si>
+  <si>
+    <t>6478889999</t>
+  </si>
+  <si>
+    <t>PreferredLanguage</t>
+  </si>
+  <si>
+    <t>EmployerPhone</t>
   </si>
 </sst>
 </file>
@@ -95,8 +216,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -377,15 +499,49 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33828E7C-EAC4-4C86-87E0-3EB8DC303443}">
+  <dimension ref="A1:AB2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="28" max="29" width="16.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -395,27 +551,157 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>46</v>
+      </c>
+      <c r="P1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1" t="s">
+        <v>16</v>
+      </c>
+      <c r="S1" t="s">
+        <v>17</v>
+      </c>
+      <c r="T1" t="s">
+        <v>18</v>
+      </c>
+      <c r="U1" t="s">
+        <v>19</v>
+      </c>
+      <c r="V1" t="s">
+        <v>20</v>
+      </c>
+      <c r="W1" t="s">
+        <v>47</v>
+      </c>
+      <c r="X1" t="s">
+        <v>21</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
+        <v>27</v>
+      </c>
+      <c r="D2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J2" t="s">
+        <v>33</v>
+      </c>
+      <c r="K2" t="s">
+        <v>34</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="M2" t="s">
+        <v>36</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="O2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>39</v>
+      </c>
+      <c r="R2" t="s">
+        <v>40</v>
+      </c>
+      <c r="S2" t="s">
+        <v>41</v>
+      </c>
+      <c r="T2" t="s">
+        <v>42</v>
+      </c>
+      <c r="U2" t="s">
+        <v>43</v>
+      </c>
+      <c r="V2" t="s">
+        <v>44</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="X2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>40</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>